<commit_message>
Apply design-review fixes; keep servo+ball valve (coarse control)
- config: sensor.type -> voltage_divider (0.5-4.5V sensor into ADS1115 3.3V + divider)
- config: tolerance_pct 2 -> 10 (ball valve is coarse; sequencer would never collect at 2%)
- BOM: remove 4-20mA-only 0.1% shunt; add fittings + electrical fixes from the audit
  (G1/4<->NPT adapter, tees, barbs, clamps, PTFE, barrel-jack pigtail, fuse,
   upstream needle valve, mount hardware, wire, bulk caps)
- README: 'Build review' section (thread mismatch, ADS wiring, MOSFET pulldown,
  bleed authority, coarse-control note, static valve-authority first test)
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -447,17 +447,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="50" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="46" customWidth="1" min="8" max="8"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -534,7 +534,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Turns the bleed valve</t>
+          <t>Turns the bleed valve (coarse control)</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>90° travel matches the servo</t>
+          <t>On/off-ish curve -&gt; coarse only</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Servo↔valve coupling bracket</t>
+          <t>Servo↔valve coupling + servo mount</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -602,7 +602,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Printed by user; servo horn comes with the servo. Optional 25T coupler (B0FLXTKGWZ, ~$8) if the design needs it</t>
+          <t>Printed; must also fix the servo BODY to react torque</t>
         </is>
       </c>
     </row>
@@ -638,7 +638,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Powers the servo off 12V, NOT the Pi rail</t>
+          <t>Powers servo off 12V, NOT the Pi</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>VERIFY 15 PSI / 100 kPa range</t>
+          <t>VERIFY 0-15 PSI / 100 kPa on the body</t>
         </is>
       </c>
     </row>
@@ -746,7 +746,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Pi has no analog input</t>
+          <t>Power at 3.3V; sensor via 10k/20k divider</t>
         </is>
       </c>
     </row>
@@ -782,7 +782,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Gate resistor + divider</t>
+          <t>Divider + MOSFET gate + pulldown come from here</t>
         </is>
       </c>
     </row>
@@ -818,7 +818,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Drives the 3-way diverter solenoid</t>
+          <t>Drives the 3-way diverter; add 10k gate pulldown</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Flyback for the solenoid</t>
+          <t>Flyback across the solenoid</t>
         </is>
       </c>
     </row>
@@ -890,7 +890,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>System 12V (valve + UBEC)</t>
+          <t>Feeds solenoid + UBEC</t>
         </is>
       </c>
     </row>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hose barb fitting kit (1/4")</t>
+          <t>Hose barb fitting kit (barb-to-barb)</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -1024,31 +1024,35 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>For tubing joins (NOT for threaded valves)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Order separately (not Amazon)</t>
+          <t>Fittings &amp; fixes (from audit)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>3-way 12V solenoid valve for WATER (diverter)</t>
+          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>53</v>
+        <v>8</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>ESValves</t>
+          <t>Amazon</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -1058,67 +1062,441 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>Amazon 3-way valves are air/gas only</t>
+          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Takeoffs for sensor + bleed branch</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1/4" NPT-M × 1/4" barb adapter</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>9.799999999999999</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Reach the silicone at every valve/sensor port</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>PTFE thread-seal tape (roll)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Hose clamps (worm/Oetiker, ~10)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Every barb-to-silicone joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>ONLY way to land the 12V into the breadboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Inline blade-fuse holder + 3A fuse</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G23" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Fire safety on the 12V behind the MOSFET</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Manual needle valve 1/4" (upstream restrictor)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Gives the bleed real authority (topology fix)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>M3 screws/standoffs + baseplate</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G25" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Mount Pi/ADS/servo bracket</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>22AWG stranded hookup wire (spool)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Reach solenoid/servo/12V</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Electrolytic caps 1000µF + 470µF</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G27" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Rail stability (UBEC out + 12V in)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
           <t>Order separately (not Amazon)</t>
         </is>
       </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>150 Ω 0.1% precision resistor (YAGEO MFP-25BRD52-150R)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>DigiKey</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Only if using the 4–20 mA sensor</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="5" t="inlineStr">
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>3-way 12V solenoid valve for WATER (diverter)</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>ESValves</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Amazon 3-way valves are air/gas only</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="5" t="inlineStr">
         <is>
           <t>TOTAL (USD)</t>
         </is>
       </c>
-      <c r="E20" s="6" t="n">
-        <v>225.75</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>You already own the Raspberry Pi 4 + microSD. Subtract $10 if you also have the USB-C PSU.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="7" t="inlineStr">
-        <is>
-          <t>Servo↔valve bracket is 3D-printed in-house (Printables: 'servo ball valve bracket').</t>
+      <c r="E30" s="6" t="n">
+        <v>308.8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. Permeability k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>MUST verify the transducer body reads 0–15 PSI (0–100 kPa). ADS1115 at 3.3V + 10k/20k divider; MOSFET needs a 10k gate pulldown (both from the resistor kit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="7" t="inlineStr">
+        <is>
+          <t>Servo coupling + servo mount are 3D-printed in-house. You already own: Pi 4, microSD, graduated cylinder.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>FIRST TEST once assembled: static valve-authority sweep (move valve full stroke, log pressure) BEFORE tuning PID.</t>
         </is>
       </c>
     </row>
@@ -1140,6 +1518,16 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G22" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId26"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sim compressor cycling + BOM additions (in-place edit)
- plant_sim: sinusoidal supply wobble (sim.supply_wobble / supply_wobble_period_s)
  models the real compressor kicking on/off; verified the PID rejects a +/-8 kPa
  supply swing (pressure held ~+/-1 kPa, 100% in-band at 20/40/60 kPa)
- BOM: 3rd tee (relief valve), 0-15 PSI dial gauge (transducer cross-check),
  splash enclosure, zip ties/heat-shrink; OPTIONAL feed-forward group
  (2nd supply-side transducer + adapter) if compressor swings beat the PID
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -43,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -73,12 +78,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -447,17 +455,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
     <col width="50" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -933,12 +941,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Fluidics &amp; proto</t>
+          <t>Sensing &amp; electronics</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Solderless breadboard 830 + jumper kit</t>
+          <t>Analog dial pressure gauge 0–15 PSI, 1/4" NPT</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -960,7 +968,11 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>NEW: cross-check / 2-point calibration of the transducer</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -970,17 +982,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Silicone tubing 1/4" ID</t>
+          <t>Solderless breadboard 830 + jumper kit</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1002,17 +1014,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Hose barb fitting kit (barb-to-barb)</t>
+          <t>Silicone tubing 1/4" ID</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1024,31 +1036,27 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>For tubing joins (NOT for threaded valves)</t>
-        </is>
-      </c>
+      <c r="H16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Fittings &amp; fixes (from audit)</t>
+          <t>Fluidics &amp; proto</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
+          <t>Hose barb fitting kit (barb-to-barb)</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1062,7 +1070,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
+          <t>For tubing joins (NOT for threaded valves)</t>
         </is>
       </c>
     </row>
@@ -1074,17 +1082,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
+          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1098,7 +1106,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Takeoffs for sensor + bleed branch</t>
+          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
         </is>
       </c>
     </row>
@@ -1110,17 +1118,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1/4" NPT-M × 1/4" barb adapter</t>
+          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>1.4</v>
+        <v>6</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>9.799999999999999</v>
+        <v>18</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1134,7 +1142,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>Reach the silicone at every valve/sensor port</t>
+          <t>NOW 3: sensor + bleed branch + relief valve</t>
         </is>
       </c>
     </row>
@@ -1146,17 +1154,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>PTFE thread-seal tape (roll)</t>
+          <t>1/4" NPT-M × 1/4" barb adapter</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>2</v>
+        <v>9.799999999999999</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1170,7 +1178,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
+          <t>Reach the silicone at every valve/sensor port</t>
         </is>
       </c>
     </row>
@@ -1182,17 +1190,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>Hose clamps (worm/Oetiker, ~10)</t>
+          <t>PTFE thread-seal tape (roll)</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1206,7 +1214,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>Every barb-to-silicone joint</t>
+          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
         </is>
       </c>
     </row>
@@ -1218,17 +1226,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
+          <t>Hose clamps (worm/Oetiker, ~10)</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1242,7 +1250,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>ONLY way to land the 12V into the breadboard</t>
+          <t>Every barb-to-silicone joint</t>
         </is>
       </c>
     </row>
@@ -1254,7 +1262,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Inline blade-fuse holder + 3A fuse</t>
+          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1278,7 +1286,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>Fire safety on the 12V behind the MOSFET</t>
+          <t>ONLY way to land the 12V into the breadboard</t>
         </is>
       </c>
     </row>
@@ -1290,17 +1298,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Manual needle valve 1/4" (upstream restrictor)</t>
+          <t>Inline blade-fuse holder + 3A fuse</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1314,7 +1322,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Gives the bleed real authority (topology fix)</t>
+          <t>Fire safety on the 12V behind the MOSFET</t>
         </is>
       </c>
     </row>
@@ -1326,17 +1334,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>M3 screws/standoffs + baseplate</t>
+          <t>Manual needle valve 1/4" (upstream restrictor)</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1350,7 +1358,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Mount Pi/ADS/servo bracket</t>
+          <t>Gives the bleed authority + attenuates compressor swings</t>
         </is>
       </c>
     </row>
@@ -1362,17 +1370,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>22AWG stranded hookup wire (spool)</t>
+          <t>M3 screws/standoffs + baseplate</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1386,7 +1394,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Reach solenoid/servo/12V</t>
+          <t>Mount Pi/ADS/servo bracket</t>
         </is>
       </c>
     </row>
@@ -1398,17 +1406,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Electrolytic caps 1000µF + 470µF</t>
+          <t>22AWG stranded hookup wire (spool)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1422,81 +1430,285 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Rail stability (UBEC out + 12V in)</t>
+          <t>Reach solenoid/servo/12V</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Electrolytic caps 1000µF + 470µF</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Rail stability (UBEC out + 12V in)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Project enclosure / splash box for electronics</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>NEW: water rig + electronics = protect the Pi/breadboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>Fittings &amp; fixes (from audit)</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Zip ties + heat-shrink assortment</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>NEW: strain relief + insulate solenoid/servo splices</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
           <t>Order separately (not Amazon)</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B31" s="2" t="inlineStr">
         <is>
           <t>3-way 12V solenoid valve for WATER (diverter)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="3" t="n">
+      <c r="C31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E31" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>ESValves</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="G31" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Amazon 3-way valves are air/gas only</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL (USD)</t>
-        </is>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>308.8</v>
-      </c>
-    </row>
     <row r="32">
-      <c r="B32" s="7" t="inlineStr">
-        <is>
-          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. Permeability k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F32" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G32" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr">
+        <is>
+          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>MUST verify the transducer body reads 0–15 PSI (0–100 kPa). ADS1115 at 3.3V + 10k/20k divider; MOSFET needs a 10k gate pulldown (both from the resistor kit).</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="7" t="inlineStr">
-        <is>
-          <t>Servo coupling + servo mount are 3D-printed in-house. You already own: Pi 4, microSD, graduated cylinder.</t>
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G33" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Mount for the supply-side sensor</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>FIRST TEST once assembled: static valve-authority sweep (move valve full stroke, log pressure) BEFORE tuning PID.</t>
+      <c r="B35" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL required (USD)</t>
+        </is>
+      </c>
+      <c r="E35" s="9" t="n">
+        <v>346.8</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL with optional (USD)</t>
+        </is>
+      </c>
+      <c r="E36" s="9" t="n">
+        <v>369.8</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="10" t="inlineStr">
+        <is>
+          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="10" t="inlineStr">
+        <is>
+          <t>The PID auto-regulates against compressor cycling (verified in sim: supply ±8 kPa -&gt; pressure held ±1 kPa, 100% in-band).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="10" t="inlineStr">
+        <is>
+          <t>OPTIONAL rows (yellow): buy only if the real compressor swing beats the PID -&gt; supply-side sensor enables feed-forward.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="10" t="inlineStr">
+        <is>
+          <t>Verify transducer body says 0–15 PSI. ADS1115 at 3.3V + 10k/20k divider. MOSFET needs 10k gate pulldown (from resistor kit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>You already own: Pi 4, microSD, graduated cylinder. Servo coupling + mount are 3D-printed in-house.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>FIRST TEST once assembled: static valve-authority sweep BEFORE tuning PID.</t>
         </is>
       </c>
     </row>
@@ -1528,6 +1740,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BOM: user owns dial gauge (removed); Pi enclosure now in-house 3D print ($0)
Required total $346.80 -> $322.80
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -610,7 +610,7 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Printed; must also fix the servo BODY to react torque</t>
+          <t>Printed by user; must fix the servo BODY to react torque</t>
         </is>
       </c>
     </row>
@@ -941,12 +941,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Sensing &amp; electronics</t>
+          <t>Fluidics &amp; proto</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Analog dial pressure gauge 0–15 PSI, 1/4" NPT</t>
+          <t>Solderless breadboard 830 + jumper kit</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -968,11 +968,7 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>NEW: cross-check / 2-point calibration of the transducer</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -982,17 +978,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Solderless breadboard 830 + jumper kit</t>
+          <t>Silicone tubing 1/4" ID</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1014,17 +1010,17 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Silicone tubing 1/4" ID</t>
+          <t>Hose barb fitting kit (barb-to-barb)</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D16" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -1036,27 +1032,31 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>For tubing joins (NOT for threaded valves)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Fluidics &amp; proto</t>
+          <t>Fittings &amp; fixes (from audit)</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Hose barb fitting kit (barb-to-barb)</t>
+          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>For tubing joins (NOT for threaded valves)</t>
+          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
         </is>
       </c>
     </row>
@@ -1082,17 +1082,17 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
+          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D18" s="3" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
+          <t>Sensor + bleed branch + relief valve</t>
         </is>
       </c>
     </row>
@@ -1118,17 +1118,17 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
+          <t>1/4" NPT-M × 1/4" barb adapter</t>
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="D19" s="3" t="n">
-        <v>6</v>
+        <v>1.4</v>
       </c>
       <c r="E19" s="3" t="n">
-        <v>18</v>
+        <v>9.799999999999999</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>NOW 3: sensor + bleed branch + relief valve</t>
+          <t>Reach the silicone at every valve/sensor port</t>
         </is>
       </c>
     </row>
@@ -1154,17 +1154,17 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>1/4" NPT-M × 1/4" barb adapter</t>
+          <t>PTFE thread-seal tape (roll)</t>
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D20" s="3" t="n">
-        <v>1.4</v>
+        <v>2</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>9.799999999999999</v>
+        <v>2</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1178,7 +1178,7 @@
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>Reach the silicone at every valve/sensor port</t>
+          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
         </is>
       </c>
     </row>
@@ -1190,17 +1190,17 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>PTFE thread-seal tape (roll)</t>
+          <t>Hose clamps (worm/Oetiker, ~10)</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1214,7 +1214,7 @@
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
+          <t>Every barb-to-silicone joint</t>
         </is>
       </c>
     </row>
@@ -1226,17 +1226,17 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Hose clamps (worm/Oetiker, ~10)</t>
+          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
         </is>
       </c>
       <c r="C22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D22" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1250,7 +1250,7 @@
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>Every barb-to-silicone joint</t>
+          <t>ONLY way to land the 12V into the breadboard</t>
         </is>
       </c>
     </row>
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
+          <t>Inline blade-fuse holder + 3A fuse</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
@@ -1286,7 +1286,7 @@
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>ONLY way to land the 12V into the breadboard</t>
+          <t>Fire safety on the 12V behind the MOSFET</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1298,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Inline blade-fuse holder + 3A fuse</t>
+          <t>Manual needle valve 1/4" (upstream restrictor)</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Fire safety on the 12V behind the MOSFET</t>
+          <t>Gives the bleed authority + attenuates compressor swings</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1334,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>Manual needle valve 1/4" (upstream restrictor)</t>
+          <t>M3 screws/standoffs + baseplate</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Gives the bleed authority + attenuates compressor swings</t>
+          <t>Mount Pi/ADS/servo bracket</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1370,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>M3 screws/standoffs + baseplate</t>
+          <t>22AWG stranded hookup wire (spool)</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Mount Pi/ADS/servo bracket</t>
+          <t>Reach solenoid/servo/12V</t>
         </is>
       </c>
     </row>
@@ -1406,17 +1406,17 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>22AWG stranded hookup wire (spool)</t>
+          <t>Electrolytic caps 1000µF + 470µF</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1430,7 +1430,7 @@
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Reach solenoid/servo/12V</t>
+          <t>Rail stability (UBEC out + 12V in)</t>
         </is>
       </c>
     </row>
@@ -1442,31 +1442,27 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Electrolytic caps 1000µF + 470µF</t>
+          <t>Pi/electronics enclosure (splash protection)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
+          <t>In-house 3D print</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr"/>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Rail stability (UBEC out + 12V in)</t>
+          <t>Designed &amp; printed by user</t>
         </is>
       </c>
     </row>
@@ -1478,17 +1474,17 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Project enclosure / splash box for electronics</t>
+          <t>Zip ties + heat-shrink assortment</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1502,33 +1498,33 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>NEW: water rig + electronics = protect the Pi/breadboard</t>
+          <t>Strain relief + insulate solenoid/servo splices</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>Fittings &amp; fixes (from audit)</t>
+          <t>Order separately (not Amazon)</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>Zip ties + heat-shrink assortment</t>
+          <t>3-way 12V solenoid valve for WATER (diverter)</t>
         </is>
       </c>
       <c r="C30" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D30" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>ESValves</t>
         </is>
       </c>
       <c r="G30" s="4" t="inlineStr">
@@ -1538,43 +1534,43 @@
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>NEW: strain relief + insulate solenoid/servo splices</t>
+          <t>Amazon 3-way valves are air/gas only</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>Order separately (not Amazon)</t>
-        </is>
-      </c>
-      <c r="B31" s="2" t="inlineStr">
-        <is>
-          <t>3-way 12V solenoid valve for WATER (diverter)</t>
-        </is>
-      </c>
-      <c r="C31" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="E31" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="F31" s="2" t="inlineStr">
-        <is>
-          <t>ESValves</t>
-        </is>
-      </c>
-      <c r="G31" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>Amazon 3-way valves are air/gas only</t>
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G31" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
         </is>
       </c>
     </row>
@@ -1586,17 +1582,17 @@
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
         </is>
       </c>
       <c r="C32" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
@@ -1610,64 +1606,35 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>OPTIONAL — feed-forward upgrade</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D33" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E33" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F33" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H33" s="5" t="inlineStr">
-        <is>
           <t>Mount for the supply-side sensor</t>
         </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL required (USD)</t>
+        </is>
+      </c>
+      <c r="E34" s="9" t="n">
+        <v>322.8</v>
       </c>
     </row>
     <row r="35">
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>TOTAL required (USD)</t>
+          <t>TOTAL with optional (USD)</t>
         </is>
       </c>
       <c r="E35" s="9" t="n">
-        <v>346.8</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL with optional (USD)</t>
-        </is>
-      </c>
-      <c r="E36" s="9" t="n">
-        <v>369.8</v>
+        <v>345.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="10" t="inlineStr">
+        <is>
+          <t>Already owned / made in-house: Pi 4, microSD, graduated cylinder, DIAL GAUGE, Pi enclosure (user-designed 3D print), servo coupling+mount.</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1701,14 +1668,7 @@
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>You already own: Pi 4, microSD, graduated cylinder. Servo coupling + mount are 3D-printed in-house.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>FIRST TEST once assembled: static valve-authority sweep BEFORE tuning PID.</t>
+          <t>FIRST TEST once assembled: static valve-authority sweep BEFORE tuning PID. Use the dial gauge for a 2-point transducer calibration.</t>
         </is>
       </c>
     </row>
@@ -1739,12 +1699,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G33" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Inline-throttle topology: single feed valve, drop needle restrictor + bleed tee
The high-flow mesh membrane + inline valve already form a pressure divider
(the manual rig regulates the same way). Command sense now topology-aware:
0% = lowest pressure (inline: closed). BOM v5: $322.80 -> $304.80
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -513,7 +513,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Servo control</t>
+          <t>Válvula de control (inline)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -542,14 +542,14 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Turns the bleed valve (coarse control)</t>
+          <t>Turns the INLINE feed valve; 0%=closed=no pressure</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Servo control</t>
+          <t>Válvula de control (inline)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -578,14 +578,14 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>On/off-ish curve -&gt; coarse only</t>
+          <t>Single valve in the feed line (like the manual rig)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Servo control</t>
+          <t>Válvula de control (inline)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -617,7 +617,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Servo control</t>
+          <t>Válvula de control (inline)</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
@@ -1086,13 +1086,13 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>6</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1106,7 +1106,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>Sensor + bleed branch + relief valve</t>
+          <t>Relief valve + spare (sensor fallback)</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1298,17 @@
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>Manual needle valve 1/4" (upstream restrictor)</t>
+          <t>M3 screws/standoffs + baseplate</t>
         </is>
       </c>
       <c r="C24" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1322,7 +1322,7 @@
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>Gives the bleed authority + attenuates compressor swings</t>
+          <t>Mount Pi/ADS/servo bracket</t>
         </is>
       </c>
     </row>
@@ -1334,17 +1334,17 @@
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>M3 screws/standoffs + baseplate</t>
+          <t>22AWG stranded hookup wire (spool)</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1358,7 +1358,7 @@
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>Mount Pi/ADS/servo bracket</t>
+          <t>Reach solenoid/servo/12V</t>
         </is>
       </c>
     </row>
@@ -1370,17 +1370,17 @@
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>22AWG stranded hookup wire (spool)</t>
+          <t>Electrolytic caps 1000µF + 470µF</t>
         </is>
       </c>
       <c r="C26" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E26" s="3" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>Reach solenoid/servo/12V</t>
+          <t>Rail stability (UBEC out + 12V in)</t>
         </is>
       </c>
     </row>
@@ -1406,31 +1406,27 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>Electrolytic caps 1000µF + 470µF</t>
+          <t>Pi/electronics enclosure (splash protection)</t>
         </is>
       </c>
       <c r="C27" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D27" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E27" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
+          <t>In-house 3D print</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>Rail stability (UBEC out + 12V in)</t>
+          <t>Designed &amp; printed by user</t>
         </is>
       </c>
     </row>
@@ -1442,53 +1438,57 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Pi/electronics enclosure (splash protection)</t>
+          <t>Zip ties + heat-shrink assortment</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>In-house 3D print</t>
-        </is>
-      </c>
-      <c r="G28" s="2" t="inlineStr"/>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Designed &amp; printed by user</t>
+          <t>Strain relief + insulate solenoid/servo splices</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>Fittings &amp; fixes (from audit)</t>
+          <t>Order separately (not Amazon)</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>Zip ties + heat-shrink assortment</t>
+          <t>3-way 12V solenoid valve for WATER (diverter)</t>
         </is>
       </c>
       <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D29" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>ESValves</t>
         </is>
       </c>
       <c r="G29" s="4" t="inlineStr">
@@ -1498,43 +1498,43 @@
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Strain relief + insulate solenoid/servo splices</t>
+          <t>Amazon 3-way valves are air/gas only</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>Order separately (not Amazon)</t>
-        </is>
-      </c>
-      <c r="B30" s="2" t="inlineStr">
-        <is>
-          <t>3-way 12V solenoid valve for WATER (diverter)</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="F30" s="2" t="inlineStr">
-        <is>
-          <t>ESValves</t>
-        </is>
-      </c>
-      <c r="G30" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>Amazon 3-way valves are air/gas only</t>
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="F30" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G30" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H30" s="5" t="inlineStr">
+        <is>
+          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
         </is>
       </c>
     </row>
@@ -1546,17 +1546,17 @@
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
         </is>
       </c>
       <c r="C31" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
@@ -1570,105 +1570,83 @@
       </c>
       <c r="H31" s="5" t="inlineStr">
         <is>
-          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
-        <is>
-          <t>OPTIONAL — feed-forward upgrade</t>
-        </is>
-      </c>
-      <c r="B32" s="5" t="inlineStr">
-        <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
-        </is>
-      </c>
-      <c r="C32" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D32" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E32" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F32" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G32" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
           <t>Mount for the supply-side sensor</t>
         </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL required (USD)</t>
+        </is>
+      </c>
+      <c r="E33" s="9" t="n">
+        <v>304.8</v>
       </c>
     </row>
     <row r="34">
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>TOTAL required (USD)</t>
+          <t>TOTAL with optional (USD)</t>
         </is>
       </c>
       <c r="E34" s="9" t="n">
-        <v>322.8</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL with optional (USD)</t>
-        </is>
-      </c>
-      <c r="E35" s="9" t="n">
-        <v>345.8</v>
+        <v>327.8</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="10" t="inlineStr">
+        <is>
+          <t>TOPOLOGY: ONE inline valve in the feed line (like the manual rig). 0% = closed = no pressure; 100% = open. No bleed/needle pair needed:</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>Already owned / made in-house: Pi 4, microSD, graduated cylinder, DIAL GAUGE, Pi enclosure (user-designed 3D print), servo coupling+mount.</t>
+          <t>the high-flow mesh membrane + the valve already form the pressure divider.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="10" t="inlineStr">
         <is>
-          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
+          <t>Already owned / made in-house: Pi 4, microSD, graduated cylinder, DIAL GAUGE, Pi enclosure (3D print), servo coupling+mount.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="10" t="inlineStr">
         <is>
-          <t>The PID auto-regulates against compressor cycling (verified in sim: supply ±8 kPa -&gt; pressure held ±1 kPa, 100% in-band).</t>
+          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="10" t="inlineStr">
         <is>
-          <t>OPTIONAL rows (yellow): buy only if the real compressor swing beats the PID -&gt; supply-side sensor enables feed-forward.</t>
+          <t>The PID auto-regulates against compressor cycling (verified in sim: supply ±8 kPa -&gt; pressure held ±1 kPa, 100% in-band).</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" s="10" t="inlineStr">
         <is>
-          <t>Verify transducer body says 0–15 PSI. ADS1115 at 3.3V + 10k/20k divider. MOSFET needs 10k gate pulldown (from resistor kit).</t>
+          <t>OPTIONAL rows (yellow): only if the real compressor swing beats the PID -&gt; supply-side sensor enables feed-forward.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" s="10" t="inlineStr">
         <is>
-          <t>FIRST TEST once assembled: static valve-authority sweep BEFORE tuning PID. Use the dial gauge for a 2-point transducer calibration.</t>
+          <t>Verify transducer body says 0–15 PSI. ADS1115 at 3.3V + 10k/20k divider. MOSFET needs 10k gate pulldown (from resistor kit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="10" t="inlineStr">
+        <is>
+          <t>FIRST TEST once assembled: sweep the servo across its travel and log pressure (valve-authority map) BEFORE tuning PID.</t>
         </is>
       </c>
     </row>
@@ -1698,11 +1676,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId27"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G32" r:id="rId29"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Real rig (photo): air-over-water, servo on EXISTING needle valve, Swagelok not NPT
- Source is compressed air; servo actuates the existing SS air needle valve
  (drop the new ball valve). Config valve comments updated for air/gas + partial
  servo range on a multi-turn needle.
- Sensor confirmed 0-15 PSI (max test ~60 kPa); range_max 100 -> 103.4 kPa;
  voltage_divider front-end. Water bath 20C -> mu=1.0e-3 (already default).
- Plumbing is Swagelok/compression: BOM fittings group flagged 'measure tube OD',
  transducer to mount at existing manometer port; relief may be redundant with
  the gas panel. Total $304.80 -> $292.20
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -43,7 +43,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -53,6 +53,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002F5597"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
       </patternFill>
     </fill>
     <fill>
@@ -78,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -87,6 +92,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -455,17 +463,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H43"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="52" customWidth="1" min="2" max="2"/>
     <col width="6" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="58" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -513,7 +521,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Válvula de control (inline)</t>
+          <t>Control (air line, on existing valve)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -542,97 +550,97 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Turns the INLINE feed valve; 0%=closed=no pressure</t>
+          <t>Turns the EXISTING SS air needle valve</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Válvula de control (inline)</t>
+          <t>Control (air line, on existing valve)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1/4" brass quarter-turn ball valve, lever</t>
+          <t>Servo↔needle-valve coupling + servo mount</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
+          <t>In-house 3D print</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Single valve in the feed line (like the manual rig)</t>
+          <t>Printed by you, onto the existing green needle-valve knob</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Válvula de control (inline)</t>
+          <t>Control (air line, on existing valve)</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Servo↔valve coupling + servo mount</t>
+          <t>UBEC 12V→6V 3A (servo power)</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="E4" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>In-house 3D print</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Printed by user; must fix the servo BODY to react torque</t>
+          <t>Powers servo off 12V, NOT the Pi</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Válvula de control (inline)</t>
+          <t>Sensing &amp; electronics</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>UBEC 12V→6V 3A (servo power)</t>
+          <t>Official Raspberry Pi 15W USB-C PSU (SC0218)</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -646,7 +654,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>Powers servo off 12V, NOT the Pi</t>
+          <t>SKIP if you already have it</t>
         </is>
       </c>
     </row>
@@ -658,17 +666,17 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Official Raspberry Pi 15W USB-C PSU (SC0218)</t>
+          <t>Pressure transducer 0–15 PSI, 0.5–4.5V, G1/4</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -682,7 +690,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>SKIP if you already have it</t>
+          <t>0-15 PSI = 0-103 kPa; tests top ~60 kPa</t>
         </is>
       </c>
     </row>
@@ -694,17 +702,17 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Pressure transducer 0–15 PSI, 0.5–4.5V, G1/4</t>
+          <t>ADS1115 16-bit I2C ADC</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -718,7 +726,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>VERIFY 0-15 PSI / 100 kPa on the body</t>
+          <t>Power at 3.3V; sensor via 10k/20k divider</t>
         </is>
       </c>
     </row>
@@ -730,17 +738,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ADS1115 16-bit I2C ADC</t>
+          <t>Resistor assortment kit (1% metal film)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -754,7 +762,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Power at 3.3V; sensor via 10k/20k divider</t>
+          <t>Divider + MOSFET gate + pulldown come from here</t>
         </is>
       </c>
     </row>
@@ -766,17 +774,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Resistor assortment kit (1% metal film)</t>
+          <t>IRLZ44N logic-level MOSFET (10-pack)</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -790,7 +798,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Divider + MOSFET gate + pulldown come from here</t>
+          <t>Drives the 3-way diverter; add 10k gate pulldown</t>
         </is>
       </c>
     </row>
@@ -802,17 +810,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>IRLZ44N logic-level MOSFET (10-pack)</t>
+          <t>1N5819 Schottky diode (100-pack)</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -826,7 +834,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Drives the 3-way diverter; add 10k gate pulldown</t>
+          <t>Flyback across the solenoid</t>
         </is>
       </c>
     </row>
@@ -838,17 +846,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1N5819 Schottky diode (100-pack)</t>
+          <t>12V 3A DC power supply (5.5×2.1mm)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -862,7 +870,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Flyback across the solenoid</t>
+          <t>Feeds solenoid + UBEC</t>
         </is>
       </c>
     </row>
@@ -874,17 +882,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>12V 3A DC power supply (5.5×2.1mm)</t>
+          <t>Adjustable relief valve CR25-100 (SAFETY)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -898,29 +906,29 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Feeds solenoid + UBEC</t>
+          <t>On the air side; SKIP if the gas panel already relieves</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Sensing &amp; electronics</t>
+          <t>Fluidics &amp; proto</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Adjustable relief valve CR25-100 (SAFETY)</t>
+          <t>Solderless breadboard 830 + jumper kit</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -932,11 +940,7 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>MANDATORY mechanical failsafe</t>
-        </is>
-      </c>
+      <c r="H13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -946,17 +950,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Solderless breadboard 830 + jumper kit</t>
+          <t>Silicone tubing 1/4" ID (permeate side)</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -968,7 +972,11 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Low-pressure permeate line only</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -978,17 +986,17 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Silicone tubing 1/4" ID</t>
+          <t>Hose barb fitting kit (barb-to-barb)</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -1000,459 +1008,463 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Permeate tubing joins</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Fluidics &amp; proto</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Hose barb fitting kit (barb-to-barb)</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="3" t="n">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Transducer adapter: G1/4-M → Swagelok (size = tube OD)</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t>McMaster/Swagelok</t>
+        </is>
+      </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr">
+        <is>
+          <t>Rig is compression/Swagelok, NOT NPT. Or mount at the existing manometer port</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Swagelok tee for sensor/relief tap (size = tube OD)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D17" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="E16" s="3" t="n">
+      <c r="E17" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>For tubing joins (NOT for threaded valves)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter w/ sealing washer</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="3" t="n">
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>McMaster/Swagelok</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>CHECK LAB STOCK first — labs with these rigs usually have bins of these</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>1/4" NPT-M × 1/4" barb adapter</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>4.199999999999999</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G18" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="inlineStr">
+        <is>
+          <t>For the 3-way diverter ports -&gt; silicone (permeate side)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>PTFE thread-seal tape (roll)</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>NPT (diverter) joints only</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>Hose clamps (worm/Oetiker, ~10)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>7</v>
+      </c>
+      <c r="F20" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G20" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="inlineStr">
+        <is>
+          <t>Every barb-to-silicone joint</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G21" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Land the 12V into the breadboard</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Inline blade-fuse holder + 3A fuse</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>6</v>
+      </c>
+      <c r="F22" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G22" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr">
+        <is>
+          <t>Fire safety on the 12V</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>M3 screws/standoffs + baseplate</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G23" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Mount Pi/ADS/servo bracket</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>22AWG stranded hookup wire (spool)</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E17" s="3" t="n">
+      <c r="E24" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>ONLY way to mount the G1/4 sensor onto NPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Brass 1/4" NPT tee (barb×barb×FNPT)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E18" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>Relief valve + spare (sensor fallback)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>1/4" NPT-M × 1/4" barb adapter</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="D19" s="3" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>9.799999999999999</v>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>Reach the silicone at every valve/sensor port</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>PTFE thread-seal tape (roll)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>NPT tapered joints only (NOT the G1/4 flat seal)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Hose clamps (worm/Oetiker, ~10)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="E21" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G21" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>Every barb-to-silicone joint</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E22" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>ONLY way to land the 12V into the breadboard</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Inline blade-fuse holder + 3A fuse</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D23" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="E23" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G23" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>Fire safety on the 12V behind the MOSFET</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>M3 screws/standoffs + baseplate</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="E24" s="3" t="n">
-        <v>10</v>
-      </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>Mount Pi/ADS/servo bracket</t>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G24" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr">
+        <is>
+          <t>Reach solenoid/servo/12V</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>22AWG stranded hookup wire (spool)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D25" s="3" t="n">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Electrolytic caps 1000µF + 470µF</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G25" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Rail stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>Pi/electronics enclosure (splash protection)</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>In-house 3D print</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="inlineStr"/>
+      <c r="H26" s="5" t="inlineStr">
+        <is>
+          <t>Designed &amp; printed by you</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Zip ties + heat-shrink assortment</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E25" s="3" t="n">
+      <c r="E27" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>Reach solenoid/servo/12V</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Electrolytic caps 1000µF + 470µF</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E26" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>Rail stability (UBEC out + 12V in)</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Fittings &amp; fixes (from audit)</t>
-        </is>
-      </c>
-      <c r="B27" s="2" t="inlineStr">
-        <is>
-          <t>Pi/electronics enclosure (splash protection)</t>
-        </is>
-      </c>
-      <c r="C27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="F27" s="2" t="inlineStr">
-        <is>
-          <t>In-house 3D print</t>
-        </is>
-      </c>
-      <c r="G27" s="2" t="inlineStr"/>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>Designed &amp; printed by user</t>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G27" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Strain relief + insulate splices</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>Fittings &amp; fixes (from audit)</t>
+          <t>Order separately (not Amazon)</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>Zip ties + heat-shrink assortment</t>
+          <t>3-way 12V solenoid valve for WATER (diverter)</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D28" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>8</v>
+        <v>53</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>ESValves</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
@@ -1462,198 +1474,162 @@
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>Strain relief + insulate solenoid/servo splices</t>
+          <t>On the permeate outlet; Amazon 3-way are air/gas only</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Order separately (not Amazon)</t>
-        </is>
-      </c>
-      <c r="B29" s="2" t="inlineStr">
-        <is>
-          <t>3-way 12V solenoid valve for WATER (diverter)</t>
-        </is>
-      </c>
-      <c r="C29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="E29" s="3" t="n">
-        <v>53</v>
-      </c>
-      <c r="F29" s="2" t="inlineStr">
-        <is>
-          <t>ESValves</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>Amazon 3-way valves are air/gas only</t>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E29" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G29" s="10" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Only if compressor swings beat the PID</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>OPTIONAL — feed-forward upgrade</t>
         </is>
       </c>
-      <c r="B30" s="5" t="inlineStr">
-        <is>
-          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
-        </is>
-      </c>
-      <c r="C30" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="E30" s="6" t="n">
-        <v>15</v>
-      </c>
-      <c r="F30" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G30" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H30" s="5" t="inlineStr">
-        <is>
-          <t>Only if compressor swings beat the PID: ADS1115 ch A1 + feed-forward</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>OPTIONAL — feed-forward upgrade</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>G1/4-F × 1/4"-NPT-M adapter (for 2nd sensor)</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D31" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="E31" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="F31" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>G1/4-M → Swagelok adapter (2nd sensor)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>10</v>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>McMaster/Swagelok</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
         <is>
           <t>Mount for the supply-side sensor</t>
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="B32" s="11" t="inlineStr">
+        <is>
+          <t>TOTAL required (USD)</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="n">
+        <v>292.2</v>
+      </c>
+    </row>
     <row r="33">
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>TOTAL required (USD)</t>
-        </is>
-      </c>
-      <c r="E33" s="9" t="n">
-        <v>304.8</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>TOTAL with optional (USD)</t>
         </is>
       </c>
-      <c r="E34" s="9" t="n">
-        <v>327.8</v>
+      <c r="E33" s="12" t="n">
+        <v>317.2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="13" t="inlineStr">
+        <is>
+          <t>RIG = air-over-water: compressed AIR pressurises the vessel. The servo turns the EXISTING stainless air NEEDLE VALVE (no new control valve).</t>
+        </is>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>TOPOLOGY: ONE inline valve in the feed line (like the manual rig). 0% = closed = no pressure; 100% = open. No bleed/needle pair needed:</t>
+      <c r="B36" s="13" t="inlineStr">
+        <is>
+          <t>Plumbing is Swagelok/COMPRESSION, not NPT. MEASURE the tube OD (caliper) before buying green-shaded fittings; many are likely in lab stock.</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>the high-flow mesh membrane + the valve already form the pressure divider.</t>
+      <c r="B37" s="13" t="inlineStr">
+        <is>
+          <t>Mount the transducer at the EXISTING manometer port if possible (already a Swagelok pressure tap on the line).</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="B38" s="10" t="inlineStr">
-        <is>
-          <t>Already owned / made in-house: Pi 4, microSD, graduated cylinder, DIAL GAUGE, Pi enclosure (3D print), servo coupling+mount.</t>
+      <c r="B38" s="13" t="inlineStr">
+        <is>
+          <t>Sensor 0-15 PSI (0-103 kPa) confirmed for &lt;=60 kPa tests. ADS1115 at 3.3V + 10k/20k divider. Water bath = 20 C -&gt; mu = 1.00e-3 (config default).</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="B39" s="10" t="inlineStr">
-        <is>
-          <t>Servo + ball valve = COARSE control (~±10–15%), NOT ±2%. k is still valid: Q is regressed vs the MEASURED mean ΔP per point.</t>
+      <c r="B39" s="13" t="inlineStr">
+        <is>
+          <t>Control is COARSE (servo trims the needle valve around the setpoint). k is still valid: Q is regressed vs the MEASURED mean pressure per point.</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="B40" s="10" t="inlineStr">
-        <is>
-          <t>The PID auto-regulates against compressor cycling (verified in sim: supply ±8 kPa -&gt; pressure held ±1 kPa, 100% in-band).</t>
+      <c r="B40" s="13" t="inlineStr">
+        <is>
+          <t>The PID auto-regulates against compressor cycling (sim: air-supply +/-8 kPa -&gt; pressure held ~+/-1 kPa). If down-regulation is slow, add a tiny fixed bleed on the air line.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>OPTIONAL rows (yellow): only if the real compressor swing beats the PID -&gt; supply-side sensor enables feed-forward.</t>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>OPTIONAL (yellow): supply-side sensor for feed-forward, only if needed.</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>Verify transducer body says 0–15 PSI. ADS1115 at 3.3V + 10k/20k divider. MOSFET needs 10k gate pulldown (from resistor kit).</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="10" t="inlineStr">
-        <is>
-          <t>FIRST TEST once assembled: sweep the servo across its travel and log pressure (valve-authority map) BEFORE tuning PID.</t>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>FIRST TEST once assembled: sweep the servo across the needle's travel and log pressure BEFORE tuning PID; use the dial gauge for a 2-point sensor cal.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId5"/>
@@ -1675,11 +1651,10 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Ambient temp (no water bath): auto-compute mu from measured water temp
- config: membrane.water_temp_c -> mu = 2.414e-5*10^(247.8/(T-140)) (Vogel);
  verified 20C=1.00e-3, 25C=8.9e-4. Rig runs at ambient (bath unused), so k now
  tracks the measured water temp instead of a fixed 20C guess.
- BOM note corrected (no water bath); parts unchanged, total stays $292.20
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -1550,6 +1550,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="B32" s="11" t="inlineStr">
         <is>
@@ -1570,6 +1571,7 @@
         <v>317.2</v>
       </c>
     </row>
+    <row r="34"/>
     <row r="35">
       <c r="B35" s="13" t="inlineStr">
         <is>
@@ -1594,7 +1596,7 @@
     <row r="38">
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Sensor 0-15 PSI (0-103 kPa) confirmed for &lt;=60 kPa tests. ADS1115 at 3.3V + 10k/20k divider. Water bath = 20 C -&gt; mu = 1.00e-3 (config default).</t>
+          <t>Sensor 0-15 PSI (0-103 kPa) confirmed for &lt;=60 kPa tests. ADS1115 at 3.3V + 10k/20k divider. AMBIENT temp (NO water bath): set membrane.water_temp_c to the measured water temp -&gt; mu auto-computed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Temperature as a test variable: DS18B20 probe + mu(T) live
- HAL TemperatureSensor (DS18B20 1-Wire real + mock); build_hal returns it.
- config temperature{source,manual_c,w1_id}; mu derived from water temp (Vogel).
- controller: slow temp poller off the PID loop; water_temp_c per CSV row;
  run-mean temp -> mu for the permeability calc; temp+mu in analysis/plot/xlsx.
- plant_sim: flow scales 1/mu so sim k is temperature-INVARIANT (0.000% 20-35C).
- BOM: DS18B20 probe -> $300.20; gen_bom.py added as BOM source.
</commit_message>
<xml_diff>
--- a/BOM.xlsx
+++ b/BOM.xlsx
@@ -738,17 +738,17 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Resistor assortment kit (1% metal film)</t>
+          <t>DS18B20 waterproof temperature probe (1-Wire)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -762,7 +762,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Divider + MOSFET gate + pulldown come from here</t>
+          <t>NEW: measures water temp -&gt; mu auto-computed. Data-&gt;GPIO4 + 4.7k pullup (from kit)</t>
         </is>
       </c>
     </row>
@@ -774,17 +774,17 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>IRLZ44N logic-level MOSFET (10-pack)</t>
+          <t>Resistor assortment kit (1% metal film)</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E9" s="3" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -798,7 +798,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>Drives the 3-way diverter; add 10k gate pulldown</t>
+          <t>Divider + MOSFET gate/pulldown + DS18B20 4.7k pullup</t>
         </is>
       </c>
     </row>
@@ -810,17 +810,17 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1N5819 Schottky diode (100-pack)</t>
+          <t>IRLZ44N logic-level MOSFET (10-pack)</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -834,7 +834,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Flyback across the solenoid</t>
+          <t>Drives the 3-way diverter; add 10k gate pulldown</t>
         </is>
       </c>
     </row>
@@ -846,17 +846,17 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>12V 3A DC power supply (5.5×2.1mm)</t>
+          <t>1N5819 Schottky diode (100-pack)</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -870,7 +870,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Feeds solenoid + UBEC</t>
+          <t>Flyback across the solenoid</t>
         </is>
       </c>
     </row>
@@ -882,17 +882,17 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Adjustable relief valve CR25-100 (SAFETY)</t>
+          <t>12V 3A DC power supply (5.5×2.1mm)</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -906,29 +906,29 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>On the air side; SKIP if the gas panel already relieves</t>
+          <t>Feeds solenoid + UBEC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Fluidics &amp; proto</t>
+          <t>Sensing &amp; electronics</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Solderless breadboard 830 + jumper kit</t>
+          <t>Adjustable relief valve CR25-100 (SAFETY)</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="3" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -940,7 +940,11 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>On the air side; SKIP if the gas panel already relieves</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -950,17 +954,17 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Silicone tubing 1/4" ID (permeate side)</t>
+          <t>Solderless breadboard 830 + jumper kit</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -972,11 +976,7 @@
           <t>link</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Low-pressure permeate line only</t>
-        </is>
-      </c>
+      <c r="H14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -986,67 +986,67 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
+          <t>Silicone tubing 1/4" ID (permeate side)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Low-pressure permeate line only</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Fluidics &amp; proto</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
           <t>Hose barb fitting kit (barb-to-barb)</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D15" s="3" t="n">
+      <c r="C16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="E15" s="3" t="n">
+      <c r="E16" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G15" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Permeate tubing joins</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
-        <is>
-          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Transducer adapter: G1/4-M → Swagelok (size = tube OD)</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D16" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="E16" s="6" t="n">
-        <v>10</v>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t>McMaster/Swagelok</t>
-        </is>
-      </c>
-      <c r="G16" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Rig is compression/Swagelok, NOT NPT. Or mount at the existing manometer port</t>
         </is>
       </c>
     </row>
@@ -1058,17 +1058,17 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>Swagelok tee for sensor/relief tap (size = tube OD)</t>
+          <t>Transducer adapter: G1/4-M → Swagelok (size = tube OD)</t>
         </is>
       </c>
       <c r="C17" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>CHECK LAB STOCK first — labs with these rigs usually have bins of these</t>
+          <t>Rig is compression/Swagelok, NOT NPT. Or mount at the existing manometer port</t>
         </is>
       </c>
     </row>
@@ -1094,21 +1094,21 @@
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>1/4" NPT-M × 1/4" barb adapter</t>
+          <t>Swagelok tee for sensor/relief tap (size = tube OD)</t>
         </is>
       </c>
       <c r="C18" s="5" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>1.4</v>
+        <v>12</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>4.199999999999999</v>
+        <v>12</v>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>Amazon</t>
+          <t>McMaster/Swagelok</t>
         </is>
       </c>
       <c r="G18" s="7" t="inlineStr">
@@ -1118,7 +1118,7 @@
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>For the 3-way diverter ports -&gt; silicone (permeate side)</t>
+          <t>CHECK LAB STOCK first</t>
         </is>
       </c>
     </row>
@@ -1130,17 +1130,17 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>PTFE thread-seal tape (roll)</t>
+          <t>1/4" NPT-M × 1/4" barb adapter</t>
         </is>
       </c>
       <c r="C19" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>2</v>
+        <v>1.4</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>2</v>
+        <v>4.199999999999999</v>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>NPT (diverter) joints only</t>
+          <t>For the 3-way diverter ports -&gt; silicone (permeate side)</t>
         </is>
       </c>
     </row>
@@ -1166,17 +1166,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>Hose clamps (worm/Oetiker, ~10)</t>
+          <t>PTFE thread-seal tape (roll)</t>
         </is>
       </c>
       <c r="C20" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
@@ -1190,7 +1190,7 @@
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Every barb-to-silicone joint</t>
+          <t>NPT (diverter) joints only</t>
         </is>
       </c>
     </row>
@@ -1202,17 +1202,17 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
+          <t>Hose clamps (worm/Oetiker, ~10)</t>
         </is>
       </c>
       <c r="C21" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
@@ -1226,7 +1226,7 @@
       </c>
       <c r="H21" s="5" t="inlineStr">
         <is>
-          <t>Land the 12V into the breadboard</t>
+          <t>Every barb-to-silicone joint</t>
         </is>
       </c>
     </row>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>Inline blade-fuse holder + 3A fuse</t>
+          <t>Barrel jack 5.5×2.1mm → screw terminal</t>
         </is>
       </c>
       <c r="C22" s="5" t="n">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>Fire safety on the 12V</t>
+          <t>Land the 12V into the breadboard</t>
         </is>
       </c>
     </row>
@@ -1274,17 +1274,17 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>M3 screws/standoffs + baseplate</t>
+          <t>Inline blade-fuse holder + 3A fuse</t>
         </is>
       </c>
       <c r="C23" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Mount Pi/ADS/servo bracket</t>
+          <t>Fire safety on the 12V</t>
         </is>
       </c>
     </row>
@@ -1310,17 +1310,17 @@
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>22AWG stranded hookup wire (spool)</t>
+          <t>M3 screws/standoffs + baseplate</t>
         </is>
       </c>
       <c r="C24" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
@@ -1334,7 +1334,7 @@
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>Reach solenoid/servo/12V</t>
+          <t>Mount Pi/ADS/servo bracket</t>
         </is>
       </c>
     </row>
@@ -1346,17 +1346,17 @@
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>Electrolytic caps 1000µF + 470µF</t>
+          <t>22AWG stranded hookup wire (spool)</t>
         </is>
       </c>
       <c r="C25" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
@@ -1370,7 +1370,7 @@
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Rail stability</t>
+          <t>Reach solenoid/servo/12V/probe</t>
         </is>
       </c>
     </row>
@@ -1382,27 +1382,31 @@
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>Pi/electronics enclosure (splash protection)</t>
+          <t>Electrolytic caps 1000µF + 470µF</t>
         </is>
       </c>
       <c r="C26" s="5" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>In-house 3D print</t>
-        </is>
-      </c>
-      <c r="G26" s="5" t="inlineStr"/>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>Designed &amp; printed by you</t>
+          <t>Rail stability</t>
         </is>
       </c>
     </row>
@@ -1414,103 +1418,99 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
+          <t>Pi/electronics enclosure (splash protection)</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>In-house 3D print</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr"/>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Designed &amp; printed by you</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>Fittings — MEASURE tube OD first (Swagelok rig)</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
           <t>Zip ties + heat-shrink assortment</t>
         </is>
       </c>
-      <c r="C27" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="D27" s="6" t="n">
+      <c r="C28" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="E27" s="6" t="n">
+      <c r="E28" s="6" t="n">
         <v>8</v>
       </c>
-      <c r="F27" s="5" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H27" s="5" t="inlineStr">
+      <c r="F28" s="5" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G28" s="7" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H28" s="5" t="inlineStr">
         <is>
           <t>Strain relief + insulate splices</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="2" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>Order separately (not Amazon)</t>
         </is>
       </c>
-      <c r="B28" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>3-way 12V solenoid valve for WATER (diverter)</t>
         </is>
       </c>
-      <c r="C28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D28" s="3" t="n">
+      <c r="C29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="E28" s="3" t="n">
+      <c r="E29" s="3" t="n">
         <v>53</v>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>ESValves</t>
         </is>
       </c>
-      <c r="G28" s="4" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="G29" s="4" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>On the permeate outlet; Amazon 3-way are air/gas only</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="8" t="inlineStr">
-        <is>
-          <t>OPTIONAL — feed-forward upgrade</t>
-        </is>
-      </c>
-      <c r="B29" s="8" t="inlineStr">
-        <is>
-          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
-        </is>
-      </c>
-      <c r="C29" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D29" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="E29" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="F29" s="8" t="inlineStr">
-        <is>
-          <t>Amazon</t>
-        </is>
-      </c>
-      <c r="G29" s="10" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H29" s="8" t="inlineStr">
-        <is>
-          <t>Only if compressor swings beat the PID</t>
         </is>
       </c>
     </row>
@@ -1522,95 +1522,122 @@
       </c>
       <c r="B30" s="8" t="inlineStr">
         <is>
+          <t>2nd pressure transducer 0–15 PSI (supply side)</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="E30" s="9" t="n">
+        <v>15</v>
+      </c>
+      <c r="F30" s="8" t="inlineStr">
+        <is>
+          <t>Amazon</t>
+        </is>
+      </c>
+      <c r="G30" s="10" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H30" s="8" t="inlineStr">
+        <is>
+          <t>Only if compressor swings beat the PID</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="8" t="inlineStr">
+        <is>
+          <t>OPTIONAL — feed-forward upgrade</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
           <t>G1/4-M → Swagelok adapter (2nd sensor)</t>
         </is>
       </c>
-      <c r="C30" s="8" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="9" t="n">
+      <c r="C31" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="E30" s="9" t="n">
+      <c r="E31" s="9" t="n">
         <v>10</v>
       </c>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F31" s="8" t="inlineStr">
         <is>
           <t>McMaster/Swagelok</t>
         </is>
       </c>
-      <c r="G30" s="10" t="inlineStr">
-        <is>
-          <t>link</t>
-        </is>
-      </c>
-      <c r="H30" s="8" t="inlineStr">
+      <c r="G31" s="10" t="inlineStr">
+        <is>
+          <t>link</t>
+        </is>
+      </c>
+      <c r="H31" s="8" t="inlineStr">
         <is>
           <t>Mount for the supply-side sensor</t>
         </is>
-      </c>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>TOTAL required (USD)</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="n">
-        <v>292.2</v>
       </c>
     </row>
     <row r="33">
       <c r="B33" s="11" t="inlineStr">
         <is>
+          <t>TOTAL required (USD)</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="n">
+        <v>300.2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="11" t="inlineStr">
+        <is>
           <t>TOTAL with optional (USD)</t>
         </is>
       </c>
-      <c r="E33" s="12" t="n">
-        <v>317.2</v>
-      </c>
-    </row>
-    <row r="34"/>
-    <row r="35">
-      <c r="B35" s="13" t="inlineStr">
-        <is>
-          <t>RIG = air-over-water: compressed AIR pressurises the vessel. The servo turns the EXISTING stainless air NEEDLE VALVE (no new control valve).</t>
-        </is>
+      <c r="E34" s="12" t="n">
+        <v>325.2</v>
       </c>
     </row>
     <row r="36">
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Plumbing is Swagelok/COMPRESSION, not NPT. MEASURE the tube OD (caliper) before buying green-shaded fittings; many are likely in lab stock.</t>
+          <t>RIG = air-over-water: compressed AIR pressurises the vessel. The servo turns the EXISTING stainless air NEEDLE VALVE (no new control valve).</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>Mount the transducer at the EXISTING manometer port if possible (already a Swagelok pressure tap on the line).</t>
+          <t>TEMPERATURE is a test variable (distilled water). The DS18B20 probe measures the water temp -&gt; the software computes mu(T) and logs it. k comes out ~constant across temperature (validation).</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Sensor 0-15 PSI (0-103 kPa) confirmed for &lt;=60 kPa tests. ADS1115 at 3.3V + 10k/20k divider. AMBIENT temp (NO water bath): set membrane.water_temp_c to the measured water temp -&gt; mu auto-computed.</t>
+          <t>Plumbing is Swagelok/COMPRESSION, not NPT. MEASURE the tube OD (caliper) before buying green-shaded fittings; many are likely in lab stock. Mount the transducer at the existing manometer port if possible.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Control is COARSE (servo trims the needle valve around the setpoint). k is still valid: Q is regressed vs the MEASURED mean pressure per point.</t>
+          <t>Sensor 0-15 PSI (0-103 kPa) for &lt;=60 kPa tests. ADS1115 at 3.3V + 10k/20k divider. DS18B20 on GPIO4 + 4.7k pullup.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>The PID auto-regulates against compressor cycling (sim: air-supply +/-8 kPa -&gt; pressure held ~+/-1 kPa). If down-regulation is slow, add a tiny fixed bleed on the air line.</t>
+          <t>Control is COARSE (servo trims the needle valve). k is still valid: Q is regressed vs the MEASURED mean pressure per point.</t>
         </is>
       </c>
     </row>
@@ -1653,10 +1680,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G23" r:id="rId21"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G24" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G25" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G27" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G26" r:id="rId24"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G28" r:id="rId25"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G29" r:id="rId26"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G30" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G31" r:id="rId28"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>